<commit_message>
Fixed additional issues with reports
</commit_message>
<xml_diff>
--- a/templates/PORT/country_data.xlsx
+++ b/templates/PORT/country_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5aee5c5b004427f/Documents/mr-risk-assessment/templates/PORT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{DFD35632-1C6F-4C62-8816-BDB3882AF2C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{244B4E1E-1E02-4CC1-AF65-7C9740683A18}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{DFD35632-1C6F-4C62-8816-BDB3882AF2C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2351DB0E-3D9A-46E0-BE59-93BBF5474980}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="773" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="773" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1-Geral" sheetId="1" r:id="rId1"/>
@@ -232,7 +232,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="101">
   <si>
     <t>Case ID</t>
   </si>
@@ -262,9 +262,6 @@
   </si>
   <si>
     <t>M</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>Year</t>
@@ -436,16 +433,7 @@
     <t>Pendiente</t>
   </si>
   <si>
-    <t>Mas de 3</t>
-  </si>
-  <si>
     <t>Desconocido</t>
-  </si>
-  <si>
-    <t>No elegible</t>
-  </si>
-  <si>
-    <t>Si</t>
   </si>
   <si>
     <t>Texto</t>
@@ -684,6 +672,41 @@
   <si>
     <t>Áreas subnacionais com uma equipe que foi treinada para resposta a surtos nos últimos 2 anos (Sim/Não)</t>
   </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>Não elegible</t>
+  </si>
+  <si>
+    <t>Mais de 3</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Não</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> elegible</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -694,7 +717,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -911,6 +934,14 @@
       <color indexed="10"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="13">
@@ -2643,21 +2674,21 @@
   <sheetData>
     <row r="1" spans="1:2" ht="30.9" customHeight="1">
       <c r="A1" s="27" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B2" s="4"/>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B3" s="4">
         <v>2024</v>
@@ -2665,42 +2696,42 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B5" s="4"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B6" s="4"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B7" s="4"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -2733,22 +2764,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="45" customHeight="1">
       <c r="A1" s="44" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B1" s="44" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F1" s="45" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2870,33 +2901,33 @@
   <sheetData>
     <row r="1" spans="1:15" ht="60.9" customHeight="1">
       <c r="A1" s="55" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B1" s="55" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C1" s="56" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E1" s="56" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F1" s="56"/>
       <c r="G1" s="56"/>
       <c r="H1" s="56"/>
       <c r="I1" s="56"/>
       <c r="J1" s="56" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="K1" s="56"/>
       <c r="L1" s="56"/>
       <c r="M1" s="56"/>
       <c r="N1" s="56"/>
       <c r="O1" s="56" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -3152,31 +3183,31 @@
   <sheetData>
     <row r="1" spans="1:9" ht="57.9" customHeight="1">
       <c r="A1" s="55" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B1" s="55" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C1" s="56" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="56" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="56" t="s">
-        <v>97</v>
-      </c>
-      <c r="E1" s="34" t="s">
+      <c r="G1" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="33" t="s">
         <v>56</v>
-      </c>
-      <c r="F1" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="H1" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="I1" s="33" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -3427,40 +3458,40 @@
   <sheetData>
     <row r="1" spans="1:12" ht="112.5" customHeight="1">
       <c r="A1" s="55" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B1" s="55" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C1" s="56" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E1" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="H1" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="K1" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="H1" s="34" t="s">
+      <c r="L1" s="34" t="s">
         <v>63</v>
-      </c>
-      <c r="I1" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="34" t="s">
-        <v>65</v>
-      </c>
-      <c r="K1" s="34" t="s">
-        <v>66</v>
-      </c>
-      <c r="L1" s="34" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="29.15" customHeight="1">
@@ -3675,7 +3706,7 @@
       <c r="D1" s="6"/>
       <c r="E1" s="9"/>
       <c r="F1" s="61" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G1" s="62"/>
       <c r="H1" s="62"/>
@@ -3698,7 +3729,7 @@
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
       <c r="F2" s="59" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G2" s="63"/>
       <c r="H2" s="63"/>
@@ -3724,7 +3755,7 @@
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
       <c r="F3" s="64" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
@@ -3747,7 +3778,7 @@
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="59" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
@@ -3770,7 +3801,7 @@
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="59" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G5" s="63"/>
       <c r="H5" s="63"/>
@@ -3793,7 +3824,7 @@
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="59" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G6" s="60"/>
       <c r="H6" s="60"/>
@@ -3874,120 +3905,120 @@
     </row>
     <row r="10" spans="1:19" ht="24">
       <c r="A10" s="15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J10" s="16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="P10" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="Q10" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="R10" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="S10" s="16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:19">
       <c r="A11" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="E11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="K11" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="L11" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="M11" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="J11" s="3" t="s">
+      <c r="N11" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="O11" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="L11" s="3" t="s">
+      <c r="P11" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="Q11" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="N11" s="3" t="s">
+      <c r="R11" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="O11" s="3" t="s">
+      <c r="S11" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="P11" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q11" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="R11" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="S11" s="3" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -4013,61 +4044,61 @@
     </row>
     <row r="13" spans="1:19">
       <c r="A13" s="18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>1</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13" s="18" t="s">
         <v>0</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H13" s="18" t="s">
         <v>3</v>
       </c>
       <c r="I13" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="K13" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="J13" s="18" t="s">
+      <c r="L13" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="M13" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="N13" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="O13" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="P13" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q13" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="R13" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="K13" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="L13" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="M13" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="N13" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="O13" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="P13" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q13" s="30" t="s">
+      <c r="S13" s="29" t="s">
         <v>24</v>
-      </c>
-      <c r="R13" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="S13" s="29" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -4092,7 +4123,7 @@
     </row>
     <row r="15" spans="1:19">
       <c r="A15" s="50" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B15" s="50"/>
       <c r="C15" s="50"/>
@@ -4699,22 +4730,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="91.65" customHeight="1">
       <c r="A1" s="31" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C1" s="37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E1" s="37" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F1" s="37" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -4852,7 +4883,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>8</v>
@@ -4861,18 +4892,18 @@
         <v>0</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>37</v>
+        <v>96</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>37</v>
+        <v>96</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>37</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>9</v>
@@ -4881,54 +4912,54 @@
         <v>1</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E4" s="8">
         <v>2</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" s="8">
         <v>3</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>36</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="E6" s="8" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="G6" s="8"/>
     </row>
     <row r="7" spans="1:11">
       <c r="E7" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="E8" s="6" t="s">
-        <v>36</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -4945,21 +4976,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007C69FE739999C447A76F1EF8B3FD66E4" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cbd048430c8551c34c2c3c8571f1b260">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="4655c133-e14e-4d88-8fbc-c3b347145ec5" xmlns:ns4="64ced670-a384-4657-ba0f-fc07d30f5a44" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5457dbb80d17598a17de4d439e456cf2" ns3:_="" ns4:_="">
     <xsd:import namespace="4655c133-e14e-4d88-8fbc-c3b347145ec5"/>
@@ -5182,32 +5198,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A51E5E2-41F2-4A1F-A4B0-950DEDB4B143}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="64ced670-a384-4657-ba0f-fc07d30f5a44"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="4655c133-e14e-4d88-8fbc-c3b347145ec5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6264E33-6917-4678-8EC8-8D88A2F9795C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1C9E008-75C3-4280-8CCC-7498B59407BC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5224,4 +5230,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6264E33-6917-4678-8EC8-8D88A2F9795C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A51E5E2-41F2-4A1F-A4B0-950DEDB4B143}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="64ced670-a384-4657-ba0f-fc07d30f5a44"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="4655c133-e14e-4d88-8fbc-c3b347145ec5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>